<commit_message>
VERTEXA biznes planı: maliyyə modelləri, pitch deck-lər, komanda planı
- VERTEXA (FEEDRATE + QUOTEFLOW + FORMCHECK + CONFIGFLOW) 2-fazalı model
- Pitch deck (.pptx), 48 aylıq maliyyə modeli (.xlsx), şirkət planı (.docx)
- Lean 12+2 komanda, ~$1M seed, FAZA 2 öz gəliri ilə
- Pessimist/baza/optimist ssenarilər, supplier + escrow + ödəniş arxitekturası

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FEEDRATE-Maliyye-Model-Premium.xlsx
+++ b/FEEDRATE-Maliyye-Model-Premium.xlsx
@@ -2816,7 +2816,7 @@
         </is>
       </c>
       <c r="B22" s="23" t="n">
-        <v>4000</v>
+        <v>10000</v>
       </c>
       <c r="C22" s="15" t="inlineStr"/>
     </row>
@@ -2838,7 +2838,7 @@
         </is>
       </c>
       <c r="B24" s="23" t="n">
-        <v>1500000</v>
+        <v>1600000</v>
       </c>
       <c r="C24" s="15" t="inlineStr">
         <is>
@@ -2853,7 +2853,7 @@
         </is>
       </c>
       <c r="B25" s="23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C25" s="15" t="inlineStr">
         <is>
@@ -3003,7 +3003,7 @@
       </c>
       <c r="S2" s="7" t="inlineStr">
         <is>
-          <t>İnzibati $</t>
+          <t>İnzibati+səyahət+bonus $</t>
         </is>
       </c>
       <c r="T2" s="7" t="inlineStr">
@@ -3099,7 +3099,7 @@
         <v>17100</v>
       </c>
       <c r="S3" s="26">
-        <f>'Fərziyyələr'!$B$23+0</f>
+        <f>'Fərziyyələr'!$B$23+0+10630</f>
         <v/>
       </c>
       <c r="T3" s="26">
@@ -3191,7 +3191,7 @@
         <v>14400</v>
       </c>
       <c r="S4" s="26">
-        <f>'Fərziyyələr'!$B$23+0</f>
+        <f>'Fərziyyələr'!$B$23+0+10069</f>
         <v/>
       </c>
       <c r="T4" s="26">
@@ -3283,7 +3283,7 @@
         <v>0</v>
       </c>
       <c r="S5" s="26">
-        <f>'Fərziyyələr'!$B$23+0</f>
+        <f>'Fərziyyələr'!$B$23+0+10077</f>
         <v/>
       </c>
       <c r="T5" s="26">
@@ -3375,7 +3375,7 @@
         <v>0</v>
       </c>
       <c r="S6" s="26">
-        <f>'Fərziyyələr'!$B$23+0</f>
+        <f>'Fərziyyələr'!$B$23+0+10085</f>
         <v/>
       </c>
       <c r="T6" s="26">
@@ -3467,7 +3467,7 @@
         <v>0</v>
       </c>
       <c r="S7" s="26">
-        <f>'Fərziyyələr'!$B$23+0</f>
+        <f>'Fərziyyələr'!$B$23+0+10095</f>
         <v/>
       </c>
       <c r="T7" s="26">
@@ -3559,7 +3559,7 @@
         <v>3500</v>
       </c>
       <c r="S8" s="26">
-        <f>'Fərziyyələr'!$B$23+0</f>
+        <f>'Fərziyyələr'!$B$23+0+10105</f>
         <v/>
       </c>
       <c r="T8" s="26">
@@ -3651,7 +3651,7 @@
         <v>0</v>
       </c>
       <c r="S9" s="26">
-        <f>'Fərziyyələr'!$B$23+0</f>
+        <f>'Fərziyyələr'!$B$23+0+3117</f>
         <v/>
       </c>
       <c r="T9" s="26">
@@ -3743,7 +3743,7 @@
         <v>0</v>
       </c>
       <c r="S10" s="26">
-        <f>'Fərziyyələr'!$B$23+0</f>
+        <f>'Fərziyyələr'!$B$23+0+3130</f>
         <v/>
       </c>
       <c r="T10" s="26">
@@ -3835,7 +3835,7 @@
         <v>1300</v>
       </c>
       <c r="S11" s="26">
-        <f>'Fərziyyələr'!$B$23+0</f>
+        <f>'Fərziyyələr'!$B$23+0+3144</f>
         <v/>
       </c>
       <c r="T11" s="26">
@@ -3927,7 +3927,7 @@
         <v>0</v>
       </c>
       <c r="S12" s="26">
-        <f>'Fərziyyələr'!$B$23+0</f>
+        <f>'Fərziyyələr'!$B$23+0+3160</f>
         <v/>
       </c>
       <c r="T12" s="26">
@@ -4019,7 +4019,7 @@
         <v>0</v>
       </c>
       <c r="S13" s="26">
-        <f>'Fərziyyələr'!$B$23+0</f>
+        <f>'Fərziyyələr'!$B$23+0+3177</f>
         <v/>
       </c>
       <c r="T13" s="26">
@@ -4111,7 +4111,7 @@
         <v>1300</v>
       </c>
       <c r="S14" s="26">
-        <f>'Fərziyyələr'!$B$23+0</f>
+        <f>'Fərziyyələr'!$B$23+0+3197</f>
         <v/>
       </c>
       <c r="T14" s="26">
@@ -4203,7 +4203,7 @@
         <v>0</v>
       </c>
       <c r="S15" s="26">
-        <f>'Fərziyyələr'!$B$23+300</f>
+        <f>'Fərziyyələr'!$B$23+300+3218</f>
         <v/>
       </c>
       <c r="T15" s="26">
@@ -4295,7 +4295,7 @@
         <v>0</v>
       </c>
       <c r="S16" s="26">
-        <f>'Fərziyyələr'!$B$23+300</f>
+        <f>'Fərziyyələr'!$B$23+300+3242</f>
         <v/>
       </c>
       <c r="T16" s="26">
@@ -4387,7 +4387,7 @@
         <v>0</v>
       </c>
       <c r="S17" s="26">
-        <f>'Fərziyyələr'!$B$23+300</f>
+        <f>'Fərziyyələr'!$B$23+300+3269</f>
         <v/>
       </c>
       <c r="T17" s="26">
@@ -4479,7 +4479,7 @@
         <v>0</v>
       </c>
       <c r="S18" s="26">
-        <f>'Fərziyyələr'!$B$23+300</f>
+        <f>'Fərziyyələr'!$B$23+300+3299</f>
         <v/>
       </c>
       <c r="T18" s="26">
@@ -4571,7 +4571,7 @@
         <v>0</v>
       </c>
       <c r="S19" s="26">
-        <f>'Fərziyyələr'!$B$23+300</f>
+        <f>'Fərziyyələr'!$B$23+300+3332</f>
         <v/>
       </c>
       <c r="T19" s="26">
@@ -4663,7 +4663,7 @@
         <v>0</v>
       </c>
       <c r="S20" s="29">
-        <f>'Fərziyyələr'!$B$23+300</f>
+        <f>'Fərziyyələr'!$B$23+300+3368</f>
         <v/>
       </c>
       <c r="T20" s="29">
@@ -4755,7 +4755,7 @@
         <v>0</v>
       </c>
       <c r="S21" s="26">
-        <f>'Fərziyyələr'!$B$23+300</f>
+        <f>'Fərziyyələr'!$B$23+300+3409</f>
         <v/>
       </c>
       <c r="T21" s="26">
@@ -4847,7 +4847,7 @@
         <v>0</v>
       </c>
       <c r="S22" s="26">
-        <f>'Fərziyyələr'!$B$23+300</f>
+        <f>'Fərziyyələr'!$B$23+300+3453</f>
         <v/>
       </c>
       <c r="T22" s="26">
@@ -4939,7 +4939,7 @@
         <v>0</v>
       </c>
       <c r="S23" s="26">
-        <f>'Fərziyyələr'!$B$23+300</f>
+        <f>'Fərziyyələr'!$B$23+300+3503</f>
         <v/>
       </c>
       <c r="T23" s="26">
@@ -5031,7 +5031,7 @@
         <v>1300</v>
       </c>
       <c r="S24" s="26">
-        <f>'Fərziyyələr'!$B$23+300</f>
+        <f>'Fərziyyələr'!$B$23+300+3559</f>
         <v/>
       </c>
       <c r="T24" s="26">
@@ -5123,7 +5123,7 @@
         <v>0</v>
       </c>
       <c r="S25" s="26">
-        <f>'Fərziyyələr'!$B$23+300</f>
+        <f>'Fərziyyələr'!$B$23+300+3620</f>
         <v/>
       </c>
       <c r="T25" s="26">
@@ -5215,7 +5215,7 @@
         <v>0</v>
       </c>
       <c r="S26" s="26">
-        <f>'Fərziyyələr'!$B$23+300</f>
+        <f>'Fərziyyələr'!$B$23+300+3688</f>
         <v/>
       </c>
       <c r="T26" s="26">
@@ -5307,7 +5307,7 @@
         <v>0</v>
       </c>
       <c r="S27" s="26">
-        <f>'Fərziyyələr'!$B$23+700</f>
+        <f>'Fərziyyələr'!$B$23+700+3764</f>
         <v/>
       </c>
       <c r="T27" s="26">
@@ -5399,7 +5399,7 @@
         <v>0</v>
       </c>
       <c r="S28" s="26">
-        <f>'Fərziyyələr'!$B$23+700</f>
+        <f>'Fərziyyələr'!$B$23+700+3848</f>
         <v/>
       </c>
       <c r="T28" s="26">
@@ -5491,7 +5491,7 @@
         <v>0</v>
       </c>
       <c r="S29" s="26">
-        <f>'Fərziyyələr'!$B$23+700</f>
+        <f>'Fərziyyələr'!$B$23+700+3941</f>
         <v/>
       </c>
       <c r="T29" s="26">
@@ -5583,7 +5583,7 @@
         <v>0</v>
       </c>
       <c r="S30" s="26">
-        <f>'Fərziyyələr'!$B$23+700</f>
+        <f>'Fərziyyələr'!$B$23+700+4045</f>
         <v/>
       </c>
       <c r="T30" s="26">
@@ -5675,7 +5675,7 @@
         <v>0</v>
       </c>
       <c r="S31" s="26">
-        <f>'Fərziyyələr'!$B$23+700</f>
+        <f>'Fərziyyələr'!$B$23+700+4160</f>
         <v/>
       </c>
       <c r="T31" s="26">
@@ -5767,7 +5767,7 @@
         <v>2200</v>
       </c>
       <c r="S32" s="26">
-        <f>'Fərziyyələr'!$B$23+700</f>
+        <f>'Fərziyyələr'!$B$23+700+4288</f>
         <v/>
       </c>
       <c r="T32" s="26">
@@ -5859,7 +5859,7 @@
         <v>0</v>
       </c>
       <c r="S33" s="26">
-        <f>'Fərziyyələr'!$B$23+700</f>
+        <f>'Fərziyyələr'!$B$23+700+4429</f>
         <v/>
       </c>
       <c r="T33" s="26">
@@ -5951,7 +5951,7 @@
         <v>0</v>
       </c>
       <c r="S34" s="26">
-        <f>'Fərziyyələr'!$B$23+700</f>
+        <f>'Fərziyyələr'!$B$23+700+4586</f>
         <v/>
       </c>
       <c r="T34" s="26">
@@ -6043,7 +6043,7 @@
         <v>0</v>
       </c>
       <c r="S35" s="26">
-        <f>'Fərziyyələr'!$B$23+700</f>
+        <f>'Fərziyyələr'!$B$23+700+4761</f>
         <v/>
       </c>
       <c r="T35" s="26">
@@ -6135,7 +6135,7 @@
         <v>0</v>
       </c>
       <c r="S36" s="26">
-        <f>'Fərziyyələr'!$B$23+700</f>
+        <f>'Fərziyyələr'!$B$23+700+4955</f>
         <v/>
       </c>
       <c r="T36" s="26">
@@ -6227,7 +6227,7 @@
         <v>0</v>
       </c>
       <c r="S37" s="26">
-        <f>'Fərziyyələr'!$B$23+700</f>
+        <f>'Fərziyyələr'!$B$23+700+5170</f>
         <v/>
       </c>
       <c r="T37" s="26">
@@ -6319,7 +6319,7 @@
         <v>0</v>
       </c>
       <c r="S38" s="29">
-        <f>'Fərziyyələr'!$B$23+700</f>
+        <f>'Fərziyyələr'!$B$23+700+5408</f>
         <v/>
       </c>
       <c r="T38" s="29">
@@ -6411,7 +6411,7 @@
         <v>0</v>
       </c>
       <c r="S39" s="26">
-        <f>'Fərziyyələr'!$B$23+700</f>
+        <f>'Fərziyyələr'!$B$23+700+5673</f>
         <v/>
       </c>
       <c r="T39" s="26">
@@ -6503,7 +6503,7 @@
         <v>0</v>
       </c>
       <c r="S40" s="26">
-        <f>'Fərziyyələr'!$B$23+700</f>
+        <f>'Fərziyyələr'!$B$23+700+5967</f>
         <v/>
       </c>
       <c r="T40" s="26">
@@ -6595,7 +6595,7 @@
         <v>0</v>
       </c>
       <c r="S41" s="26">
-        <f>'Fərziyyələr'!$B$23+700</f>
+        <f>'Fərziyyələr'!$B$23+700+6294</f>
         <v/>
       </c>
       <c r="T41" s="26">
@@ -6687,7 +6687,7 @@
         <v>0</v>
       </c>
       <c r="S42" s="26">
-        <f>'Fərziyyələr'!$B$23+700</f>
+        <f>'Fərziyyələr'!$B$23+700+6656</f>
         <v/>
       </c>
       <c r="T42" s="26">
@@ -6779,7 +6779,7 @@
         <v>0</v>
       </c>
       <c r="S43" s="26">
-        <f>'Fərziyyələr'!$B$23+700</f>
+        <f>'Fərziyyələr'!$B$23+700+7058</f>
         <v/>
       </c>
       <c r="T43" s="26">
@@ -6871,7 +6871,7 @@
         <v>0</v>
       </c>
       <c r="S44" s="26">
-        <f>'Fərziyyələr'!$B$23+700</f>
+        <f>'Fərziyyələr'!$B$23+700+7505</f>
         <v/>
       </c>
       <c r="T44" s="26">
@@ -6963,7 +6963,7 @@
         <v>0</v>
       </c>
       <c r="S45" s="26">
-        <f>'Fərziyyələr'!$B$23+700</f>
+        <f>'Fərziyyələr'!$B$23+700+8000</f>
         <v/>
       </c>
       <c r="T45" s="26">
@@ -7055,7 +7055,7 @@
         <v>0</v>
       </c>
       <c r="S46" s="26">
-        <f>'Fərziyyələr'!$B$23+700</f>
+        <f>'Fərziyyələr'!$B$23+700+8550</f>
         <v/>
       </c>
       <c r="T46" s="26">
@@ -7147,7 +7147,7 @@
         <v>0</v>
       </c>
       <c r="S47" s="26">
-        <f>'Fərziyyələr'!$B$23+700</f>
+        <f>'Fərziyyələr'!$B$23+700+9161</f>
         <v/>
       </c>
       <c r="T47" s="26">
@@ -7239,7 +7239,7 @@
         <v>0</v>
       </c>
       <c r="S48" s="26">
-        <f>'Fərziyyələr'!$B$23+700</f>
+        <f>'Fərziyyələr'!$B$23+700+9838</f>
         <v/>
       </c>
       <c r="T48" s="26">
@@ -7331,7 +7331,7 @@
         <v>0</v>
       </c>
       <c r="S49" s="26">
-        <f>'Fərziyyələr'!$B$23+700</f>
+        <f>'Fərziyyələr'!$B$23+700+10590</f>
         <v/>
       </c>
       <c r="T49" s="26">
@@ -7423,7 +7423,7 @@
         <v>0</v>
       </c>
       <c r="S50" s="29">
-        <f>'Fərziyyələr'!$B$23+700</f>
+        <f>'Fərziyyələr'!$B$23+700+11425</f>
         <v/>
       </c>
       <c r="T50" s="29">

</xml_diff>